<commit_message>
initial training evaluation done
</commit_message>
<xml_diff>
--- a/eeg_dataset.xlsx
+++ b/eeg_dataset.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q89"/>
+  <dimension ref="A1:R89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,40 +476,45 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>path_to_small_feature_vector</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>alpha</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>beta</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>theta</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>delta</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>theta_alpha_ratio</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>slowing_index</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>coherence</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>entropy</t>
         </is>
@@ -557,28 +562,33 @@
           <t>eegpt_features/features_sub-001.pt</t>
         </is>
       </c>
-      <c r="J2" t="n">
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-001.pt</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
         <v>0.02687520906659216</v>
       </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
         <v>0.02739122940895669</v>
       </c>
-      <c r="L2" t="n">
+      <c r="M2" t="n">
         <v>0.09447417409659438</v>
       </c>
-      <c r="M2" t="n">
+      <c r="N2" t="n">
         <v>0.8338514517662171</v>
       </c>
-      <c r="N2" t="n">
+      <c r="O2" t="n">
         <v>3.518668939963756</v>
       </c>
-      <c r="O2" t="n">
+      <c r="P2" t="n">
         <v>17.27261868707939</v>
       </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
         <v>0.4027393019309905</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="R2" t="n">
         <v>1.461288974242712</v>
       </c>
     </row>
@@ -624,28 +634,33 @@
           <t>eegpt_features/features_sub-002.pt</t>
         </is>
       </c>
-      <c r="J3" t="n">
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-002.pt</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
         <v>0.06395410218462962</v>
       </c>
-      <c r="K3" t="n">
+      <c r="L3" t="n">
         <v>0.03563676672580383</v>
       </c>
-      <c r="L3" t="n">
+      <c r="M3" t="n">
         <v>0.09214453175179982</v>
       </c>
-      <c r="M3" t="n">
+      <c r="N3" t="n">
         <v>0.782128225897437</v>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>1.576171945386612</v>
       </c>
-      <c r="O3" t="n">
+      <c r="P3" t="n">
         <v>9.2351970037677</v>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
         <v>0.2910845527181644</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="R3" t="n">
         <v>1.596957867215758</v>
       </c>
     </row>
@@ -691,28 +706,33 @@
           <t>eegpt_features/features_sub-003.pt</t>
         </is>
       </c>
-      <c r="J4" t="n">
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-003.pt</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
         <v>0.1066128818648855</v>
       </c>
-      <c r="K4" t="n">
+      <c r="L4" t="n">
         <v>0.02960177527170381</v>
       </c>
-      <c r="L4" t="n">
+      <c r="M4" t="n">
         <v>0.1118372300901561</v>
       </c>
-      <c r="M4" t="n">
+      <c r="N4" t="n">
         <v>0.7180804551112254</v>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>1.21807850174216</v>
       </c>
-      <c r="O4" t="n">
+      <c r="P4" t="n">
         <v>6.834359252706034</v>
       </c>
-      <c r="P4" t="n">
-        <v>0.2991986533574498</v>
-      </c>
       <c r="Q4" t="n">
+        <v>0.2991986533574499</v>
+      </c>
+      <c r="R4" t="n">
         <v>1.688180224736507</v>
       </c>
     </row>
@@ -758,28 +778,33 @@
           <t>eegpt_features/features_sub-004.pt</t>
         </is>
       </c>
-      <c r="J5" t="n">
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-004.pt</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
         <v>0.02865991618337902</v>
       </c>
-      <c r="K5" t="n">
+      <c r="L5" t="n">
         <v>0.0335218003033412</v>
       </c>
-      <c r="L5" t="n">
+      <c r="M5" t="n">
         <v>0.09651247600986819</v>
       </c>
-      <c r="M5" t="n">
+      <c r="N5" t="n">
         <v>0.8205264054946643</v>
       </c>
-      <c r="N5" t="n">
+      <c r="O5" t="n">
         <v>3.378659268996135</v>
       </c>
-      <c r="O5" t="n">
+      <c r="P5" t="n">
         <v>15.17105218353772</v>
       </c>
-      <c r="P5" t="n">
-        <v>0.3962373900968316</v>
-      </c>
       <c r="Q5" t="n">
+        <v>0.3962373900968314</v>
+      </c>
+      <c r="R5" t="n">
         <v>1.504201435959941</v>
       </c>
     </row>
@@ -825,28 +850,33 @@
           <t>eegpt_features/features_sub-005.pt</t>
         </is>
       </c>
-      <c r="J6" t="n">
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-005.pt</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
         <v>0.03298216490259213</v>
       </c>
-      <c r="K6" t="n">
+      <c r="L6" t="n">
         <v>0.03221582152492203</v>
       </c>
-      <c r="L6" t="n">
+      <c r="M6" t="n">
         <v>0.09394721210800379</v>
       </c>
-      <c r="M6" t="n">
+      <c r="N6" t="n">
         <v>0.8204942998263337</v>
       </c>
-      <c r="N6" t="n">
+      <c r="O6" t="n">
         <v>2.879508015590928</v>
       </c>
-      <c r="O6" t="n">
+      <c r="P6" t="n">
         <v>14.28145990041531</v>
       </c>
-      <c r="P6" t="n">
-        <v>0.3846703278818872</v>
-      </c>
       <c r="Q6" t="n">
+        <v>0.3846703278818871</v>
+      </c>
+      <c r="R6" t="n">
         <v>1.498544523375284</v>
       </c>
     </row>
@@ -892,28 +922,33 @@
           <t>eegpt_features/features_sub-006.pt</t>
         </is>
       </c>
-      <c r="J7" t="n">
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-006.pt</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
         <v>0.1025336966822105</v>
       </c>
-      <c r="K7" t="n">
+      <c r="L7" t="n">
         <v>0.04196908712301304</v>
       </c>
-      <c r="L7" t="n">
+      <c r="M7" t="n">
         <v>0.07812976399984346</v>
       </c>
-      <c r="M7" t="n">
+      <c r="N7" t="n">
         <v>0.7542073262739973</v>
       </c>
-      <c r="N7" t="n">
+      <c r="O7" t="n">
         <v>0.9488041832277965</v>
       </c>
-      <c r="O7" t="n">
+      <c r="P7" t="n">
         <v>6.369494755512255</v>
       </c>
-      <c r="P7" t="n">
-        <v>0.3125476059407112</v>
-      </c>
       <c r="Q7" t="n">
+        <v>0.3125476059407111</v>
+      </c>
+      <c r="R7" t="n">
         <v>1.693524993030956</v>
       </c>
     </row>
@@ -959,28 +994,33 @@
           <t>eegpt_features/features_sub-007.pt</t>
         </is>
       </c>
-      <c r="J8" t="n">
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-007.pt</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
         <v>0.03268272632870364</v>
       </c>
-      <c r="K8" t="n">
+      <c r="L8" t="n">
         <v>0.02973134116428384</v>
       </c>
-      <c r="L8" t="n">
+      <c r="M8" t="n">
         <v>0.1025693263506144</v>
       </c>
-      <c r="M8" t="n">
+      <c r="N8" t="n">
         <v>0.8140245690628765</v>
       </c>
-      <c r="N8" t="n">
+      <c r="O8" t="n">
         <v>3.141947869850041</v>
       </c>
-      <c r="O8" t="n">
+      <c r="P8" t="n">
         <v>14.75461212598112</v>
       </c>
-      <c r="P8" t="n">
-        <v>0.3735813671055683</v>
-      </c>
       <c r="Q8" t="n">
+        <v>0.3735813671055681</v>
+      </c>
+      <c r="R8" t="n">
         <v>1.488890231344489</v>
       </c>
     </row>
@@ -1026,28 +1066,33 @@
           <t>eegpt_features/features_sub-008.pt</t>
         </is>
       </c>
-      <c r="J9" t="n">
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-008.pt</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
         <v>0.0288554984209024</v>
       </c>
-      <c r="K9" t="n">
+      <c r="L9" t="n">
         <v>0.02762313711320965</v>
       </c>
-      <c r="L9" t="n">
+      <c r="M9" t="n">
         <v>0.0817703548623482</v>
       </c>
-      <c r="M9" t="n">
+      <c r="N9" t="n">
         <v>0.8455917432959016</v>
       </c>
-      <c r="N9" t="n">
+      <c r="O9" t="n">
         <v>2.875253024526024</v>
       </c>
-      <c r="O9" t="n">
+      <c r="P9" t="n">
         <v>16.48983195742976</v>
       </c>
-      <c r="P9" t="n">
-        <v>0.3678783103511706</v>
-      </c>
       <c r="Q9" t="n">
+        <v>0.3678783103511708</v>
+      </c>
+      <c r="R9" t="n">
         <v>1.466070964414019</v>
       </c>
     </row>
@@ -1093,28 +1138,33 @@
           <t>eegpt_features/features_sub-009.pt</t>
         </is>
       </c>
-      <c r="J10" t="n">
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-009.pt</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
         <v>0.07795243719540357</v>
       </c>
-      <c r="K10" t="n">
+      <c r="L10" t="n">
         <v>0.04807250729494093</v>
       </c>
-      <c r="L10" t="n">
+      <c r="M10" t="n">
         <v>0.09383212442222966</v>
       </c>
-      <c r="M10" t="n">
+      <c r="N10" t="n">
         <v>0.7516345279967416</v>
       </c>
-      <c r="N10" t="n">
+      <c r="O10" t="n">
         <v>1.261688453280849</v>
       </c>
-      <c r="O10" t="n">
+      <c r="P10" t="n">
         <v>6.910447374415305</v>
       </c>
-      <c r="P10" t="n">
+      <c r="Q10" t="n">
         <v>0.2787392887051905</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="R10" t="n">
         <v>1.702836019007651</v>
       </c>
     </row>
@@ -1160,28 +1210,33 @@
           <t>eegpt_features/features_sub-010.pt</t>
         </is>
       </c>
-      <c r="J11" t="n">
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-010.pt</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
         <v>0.03773299345147285</v>
       </c>
-      <c r="K11" t="n">
+      <c r="L11" t="n">
         <v>0.03785961504521287</v>
       </c>
-      <c r="L11" t="n">
+      <c r="M11" t="n">
         <v>0.08815361895897333</v>
       </c>
-      <c r="M11" t="n">
+      <c r="N11" t="n">
         <v>0.8166305209338796</v>
       </c>
-      <c r="N11" t="n">
+      <c r="O11" t="n">
         <v>2.452980108063002</v>
       </c>
-      <c r="O11" t="n">
+      <c r="P11" t="n">
         <v>12.49787993849469</v>
       </c>
-      <c r="P11" t="n">
+      <c r="Q11" t="n">
         <v>0.3481533956463889</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="R11" t="n">
         <v>1.536280298570764</v>
       </c>
     </row>
@@ -1227,28 +1282,33 @@
           <t>eegpt_features/features_sub-011.pt</t>
         </is>
       </c>
-      <c r="J12" t="n">
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-011.pt</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
         <v>0.06135821502321578</v>
       </c>
-      <c r="K12" t="n">
+      <c r="L12" t="n">
         <v>0.03750091307777205</v>
       </c>
-      <c r="L12" t="n">
+      <c r="M12" t="n">
         <v>0.1041764103047432</v>
       </c>
-      <c r="M12" t="n">
+      <c r="N12" t="n">
         <v>0.7605065515380304</v>
       </c>
-      <c r="N12" t="n">
+      <c r="O12" t="n">
         <v>1.910730636217637</v>
       </c>
-      <c r="O12" t="n">
+      <c r="P12" t="n">
         <v>9.654745095613434</v>
       </c>
-      <c r="P12" t="n">
-        <v>0.2736678177572249</v>
-      </c>
       <c r="Q12" t="n">
+        <v>0.2736678177572248</v>
+      </c>
+      <c r="R12" t="n">
         <v>1.671603872950103</v>
       </c>
     </row>
@@ -1294,28 +1354,33 @@
           <t>eegpt_features/features_sub-012.pt</t>
         </is>
       </c>
-      <c r="J13" t="n">
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-012.pt</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
         <v>0.04021093640858057</v>
       </c>
-      <c r="K13" t="n">
+      <c r="L13" t="n">
         <v>0.03272623499363578</v>
       </c>
-      <c r="L13" t="n">
+      <c r="M13" t="n">
         <v>0.08797242030180329</v>
       </c>
-      <c r="M13" t="n">
+      <c r="N13" t="n">
         <v>0.8195331582106951</v>
       </c>
-      <c r="N13" t="n">
+      <c r="O13" t="n">
         <v>2.303269322627755</v>
       </c>
-      <c r="O13" t="n">
+      <c r="P13" t="n">
         <v>12.78993942564317</v>
       </c>
-      <c r="P13" t="n">
+      <c r="Q13" t="n">
         <v>0.3342693394495644</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="R13" t="n">
         <v>1.515058028032545</v>
       </c>
     </row>
@@ -1361,28 +1426,33 @@
           <t>eegpt_features/features_sub-013.pt</t>
         </is>
       </c>
-      <c r="J14" t="n">
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-013.pt</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
         <v>0.03098480232631607</v>
       </c>
-      <c r="K14" t="n">
+      <c r="L14" t="n">
         <v>0.02620505093453902</v>
       </c>
-      <c r="L14" t="n">
+      <c r="M14" t="n">
         <v>0.09701230640040652</v>
       </c>
-      <c r="M14" t="n">
+      <c r="N14" t="n">
         <v>0.8272414918970348</v>
       </c>
-      <c r="N14" t="n">
+      <c r="O14" t="n">
         <v>3.203325719098979</v>
       </c>
-      <c r="O14" t="n">
+      <c r="P14" t="n">
         <v>16.4484142495333</v>
       </c>
-      <c r="P14" t="n">
-        <v>0.3652450961350498</v>
-      </c>
       <c r="Q14" t="n">
+        <v>0.36524509613505</v>
+      </c>
+      <c r="R14" t="n">
         <v>1.461299885507122</v>
       </c>
     </row>
@@ -1428,28 +1498,33 @@
           <t>eegpt_features/features_sub-014.pt</t>
         </is>
       </c>
-      <c r="J15" t="n">
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-014.pt</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
         <v>0.02705045572110325</v>
       </c>
-      <c r="K15" t="n">
+      <c r="L15" t="n">
         <v>0.03534794736448751</v>
       </c>
-      <c r="L15" t="n">
+      <c r="M15" t="n">
         <v>0.09162875903225373</v>
       </c>
-      <c r="M15" t="n">
+      <c r="N15" t="n">
         <v>0.8294720414703067</v>
       </c>
-      <c r="N15" t="n">
+      <c r="O15" t="n">
         <v>3.398369326067777</v>
       </c>
-      <c r="O15" t="n">
+      <c r="P15" t="n">
         <v>15.90122751147548</v>
       </c>
-      <c r="P15" t="n">
+      <c r="Q15" t="n">
         <v>0.3685371403204085</v>
       </c>
-      <c r="Q15" t="n">
+      <c r="R15" t="n">
         <v>1.509079081258538</v>
       </c>
     </row>
@@ -1495,28 +1570,33 @@
           <t>eegpt_features/features_sub-015.pt</t>
         </is>
       </c>
-      <c r="J16" t="n">
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-015.pt</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
         <v>0.05069697043922167</v>
       </c>
-      <c r="K16" t="n">
+      <c r="L16" t="n">
         <v>0.02795028247161552</v>
       </c>
-      <c r="L16" t="n">
+      <c r="M16" t="n">
         <v>0.08473435648736809</v>
       </c>
-      <c r="M16" t="n">
+      <c r="N16" t="n">
         <v>0.8161579270486682</v>
       </c>
-      <c r="N16" t="n">
+      <c r="O16" t="n">
         <v>1.953413420989316</v>
       </c>
-      <c r="O16" t="n">
+      <c r="P16" t="n">
         <v>12.44655676304826</v>
       </c>
-      <c r="P16" t="n">
+      <c r="Q16" t="n">
         <v>0.2994675744852552</v>
       </c>
-      <c r="Q16" t="n">
+      <c r="R16" t="n">
         <v>1.515903920910561</v>
       </c>
     </row>
@@ -1562,28 +1642,33 @@
           <t>eegpt_features/features_sub-016.pt</t>
         </is>
       </c>
-      <c r="J17" t="n">
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-016.pt</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
         <v>0.02643051625683208</v>
       </c>
-      <c r="K17" t="n">
+      <c r="L17" t="n">
         <v>0.02274542391703009</v>
       </c>
-      <c r="L17" t="n">
+      <c r="M17" t="n">
         <v>0.09220034359139662</v>
       </c>
-      <c r="M17" t="n">
+      <c r="N17" t="n">
         <v>0.8418001647700494</v>
       </c>
-      <c r="N17" t="n">
+      <c r="O17" t="n">
         <v>3.491646583701818</v>
       </c>
-      <c r="O17" t="n">
+      <c r="P17" t="n">
         <v>19.04916972873376</v>
       </c>
-      <c r="P17" t="n">
+      <c r="Q17" t="n">
         <v>0.4084639142874238</v>
       </c>
-      <c r="Q17" t="n">
+      <c r="R17" t="n">
         <v>1.412405118507688</v>
       </c>
     </row>
@@ -1629,28 +1714,33 @@
           <t>eegpt_features/features_sub-017.pt</t>
         </is>
       </c>
-      <c r="J18" t="n">
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-017.pt</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
         <v>0.03201134144884622</v>
       </c>
-      <c r="K18" t="n">
+      <c r="L18" t="n">
         <v>0.02565907062661268</v>
       </c>
-      <c r="L18" t="n">
+      <c r="M18" t="n">
         <v>0.1013951054398669</v>
       </c>
-      <c r="M18" t="n">
+      <c r="N18" t="n">
         <v>0.8223432703213607</v>
       </c>
-      <c r="N18" t="n">
+      <c r="O18" t="n">
         <v>3.203767048653085</v>
       </c>
-      <c r="O18" t="n">
+      <c r="P18" t="n">
         <v>16.11602045724818</v>
       </c>
-      <c r="P18" t="n">
+      <c r="Q18" t="n">
         <v>0.3354715863885879</v>
       </c>
-      <c r="Q18" t="n">
+      <c r="R18" t="n">
         <v>1.430125947488569</v>
       </c>
     </row>
@@ -1696,28 +1786,33 @@
           <t>eegpt_features/features_sub-018.pt</t>
         </is>
       </c>
-      <c r="J19" t="n">
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-018.pt</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
         <v>0.05574061474009669</v>
       </c>
-      <c r="K19" t="n">
+      <c r="L19" t="n">
         <v>0.04657920844467869</v>
       </c>
-      <c r="L19" t="n">
+      <c r="M19" t="n">
         <v>0.1152143184669673</v>
       </c>
-      <c r="M19" t="n">
+      <c r="N19" t="n">
         <v>0.7509368950775998</v>
       </c>
-      <c r="N19" t="n">
+      <c r="O19" t="n">
         <v>2.113494581562846</v>
       </c>
-      <c r="O19" t="n">
+      <c r="P19" t="n">
         <v>8.598173248064137</v>
       </c>
-      <c r="P19" t="n">
+      <c r="Q19" t="n">
         <v>0.2703173363143145</v>
       </c>
-      <c r="Q19" t="n">
+      <c r="R19" t="n">
         <v>1.670549370015057</v>
       </c>
     </row>
@@ -1763,28 +1858,33 @@
           <t>eegpt_features/features_sub-019.pt</t>
         </is>
       </c>
-      <c r="J20" t="n">
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-019.pt</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
         <v>0.03220411149128051</v>
       </c>
-      <c r="K20" t="n">
+      <c r="L20" t="n">
         <v>0.03496698835942356</v>
       </c>
-      <c r="L20" t="n">
+      <c r="M20" t="n">
         <v>0.08784386772046127</v>
       </c>
-      <c r="M20" t="n">
+      <c r="N20" t="n">
         <v>0.8278906849341606</v>
       </c>
-      <c r="N20" t="n">
+      <c r="O20" t="n">
         <v>2.789954551363672</v>
       </c>
-      <c r="O20" t="n">
+      <c r="P20" t="n">
         <v>14.21249762173996</v>
       </c>
-      <c r="P20" t="n">
+      <c r="Q20" t="n">
         <v>0.3717350953580081</v>
       </c>
-      <c r="Q20" t="n">
+      <c r="R20" t="n">
         <v>1.511294509340442</v>
       </c>
     </row>
@@ -1830,28 +1930,33 @@
           <t>eegpt_features/features_sub-020.pt</t>
         </is>
       </c>
-      <c r="J21" t="n">
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-020.pt</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
         <v>0.02631317425215298</v>
       </c>
-      <c r="K21" t="n">
+      <c r="L21" t="n">
         <v>0.02489275046074536</v>
       </c>
-      <c r="L21" t="n">
+      <c r="M21" t="n">
         <v>0.08354215530436196</v>
       </c>
-      <c r="M21" t="n">
+      <c r="N21" t="n">
         <v>0.848674806805487</v>
       </c>
-      <c r="N21" t="n">
+      <c r="O21" t="n">
         <v>3.201160061708316</v>
       </c>
-      <c r="O21" t="n">
+      <c r="P21" t="n">
         <v>18.45928877908028</v>
       </c>
-      <c r="P21" t="n">
-        <v>0.3937552532647421</v>
-      </c>
       <c r="Q21" t="n">
+        <v>0.3937552532647422</v>
+      </c>
+      <c r="R21" t="n">
         <v>1.385732880995879</v>
       </c>
     </row>
@@ -1897,28 +2002,33 @@
           <t>eegpt_features/features_sub-021.pt</t>
         </is>
       </c>
-      <c r="J22" t="n">
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-021.pt</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
         <v>0.03164724022985215</v>
       </c>
-      <c r="K22" t="n">
+      <c r="L22" t="n">
         <v>0.0418817597448114</v>
       </c>
-      <c r="L22" t="n">
+      <c r="M22" t="n">
         <v>0.08815530907764547</v>
       </c>
-      <c r="M22" t="n">
+      <c r="N22" t="n">
         <v>0.8200086345592545</v>
       </c>
-      <c r="N22" t="n">
+      <c r="O22" t="n">
         <v>2.838260072670377</v>
       </c>
-      <c r="O22" t="n">
+      <c r="P22" t="n">
         <v>12.66101567267104</v>
       </c>
-      <c r="P22" t="n">
-        <v>0.3653031883861499</v>
-      </c>
       <c r="Q22" t="n">
+        <v>0.36530318838615</v>
+      </c>
+      <c r="R22" t="n">
         <v>1.553365458370218</v>
       </c>
     </row>
@@ -1964,28 +2074,33 @@
           <t>eegpt_features/features_sub-022.pt</t>
         </is>
       </c>
-      <c r="J23" t="n">
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-022.pt</t>
+        </is>
+      </c>
+      <c r="K23" t="n">
         <v>0.04457893288543752</v>
       </c>
-      <c r="K23" t="n">
+      <c r="L23" t="n">
         <v>0.04005641470294803</v>
       </c>
-      <c r="L23" t="n">
+      <c r="M23" t="n">
         <v>0.1103200805877952</v>
       </c>
-      <c r="M23" t="n">
+      <c r="N23" t="n">
         <v>0.7811476975135223</v>
       </c>
-      <c r="N23" t="n">
+      <c r="O23" t="n">
         <v>2.571823449008356</v>
       </c>
-      <c r="O23" t="n">
+      <c r="P23" t="n">
         <v>10.76311672963625</v>
       </c>
-      <c r="P23" t="n">
-        <v>0.2996312124266993</v>
-      </c>
       <c r="Q23" t="n">
+        <v>0.2996312124266992</v>
+      </c>
+      <c r="R23" t="n">
         <v>1.628004924947039</v>
       </c>
     </row>
@@ -2031,28 +2146,33 @@
           <t>eegpt_features/features_sub-023.pt</t>
         </is>
       </c>
-      <c r="J24" t="n">
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-023.pt</t>
+        </is>
+      </c>
+      <c r="K24" t="n">
         <v>0.04317625316796114</v>
       </c>
-      <c r="K24" t="n">
+      <c r="L24" t="n">
         <v>0.03839872182157247</v>
       </c>
-      <c r="L24" t="n">
+      <c r="M24" t="n">
         <v>0.09488277602976847</v>
       </c>
-      <c r="M24" t="n">
+      <c r="N24" t="n">
         <v>0.8013019413548242</v>
       </c>
-      <c r="N24" t="n">
+      <c r="O24" t="n">
         <v>2.312871632858284</v>
       </c>
-      <c r="O24" t="n">
+      <c r="P24" t="n">
         <v>11.32557654305541</v>
       </c>
-      <c r="P24" t="n">
+      <c r="Q24" t="n">
         <v>0.3214730884486022</v>
       </c>
-      <c r="Q24" t="n">
+      <c r="R24" t="n">
         <v>1.644303089669983</v>
       </c>
     </row>
@@ -2098,28 +2218,33 @@
           <t>eegpt_features/features_sub-024.pt</t>
         </is>
       </c>
-      <c r="J25" t="n">
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-024.pt</t>
+        </is>
+      </c>
+      <c r="K25" t="n">
         <v>0.0375304837561774</v>
       </c>
-      <c r="K25" t="n">
+      <c r="L25" t="n">
         <v>0.02910345193939429</v>
       </c>
-      <c r="L25" t="n">
+      <c r="M25" t="n">
         <v>0.1156922167863736</v>
       </c>
-      <c r="M25" t="n">
+      <c r="N25" t="n">
         <v>0.7876920482527673</v>
       </c>
-      <c r="N25" t="n">
+      <c r="O25" t="n">
         <v>3.091604659087775</v>
       </c>
-      <c r="O25" t="n">
+      <c r="P25" t="n">
         <v>13.67661889216517</v>
       </c>
-      <c r="P25" t="n">
+      <c r="Q25" t="n">
         <v>0.3135301917765295</v>
       </c>
-      <c r="Q25" t="n">
+      <c r="R25" t="n">
         <v>1.511170328428514</v>
       </c>
     </row>
@@ -2165,28 +2290,33 @@
           <t>eegpt_features/features_sub-025.pt</t>
         </is>
       </c>
-      <c r="J26" t="n">
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-025.pt</t>
+        </is>
+      </c>
+      <c r="K26" t="n">
         <v>0.07219857323072541</v>
       </c>
-      <c r="K26" t="n">
+      <c r="L26" t="n">
         <v>0.0345114290169079</v>
       </c>
-      <c r="L26" t="n">
+      <c r="M26" t="n">
         <v>0.08419165168289015</v>
       </c>
-      <c r="M26" t="n">
+      <c r="N26" t="n">
         <v>0.7904533465033639</v>
       </c>
-      <c r="N26" t="n">
+      <c r="O26" t="n">
         <v>1.747218879130591</v>
       </c>
-      <c r="O26" t="n">
+      <c r="P26" t="n">
         <v>10.40385840759904</v>
       </c>
-      <c r="P26" t="n">
-        <v>0.3246370675502562</v>
-      </c>
       <c r="Q26" t="n">
+        <v>0.3246370675502563</v>
+      </c>
+      <c r="R26" t="n">
         <v>1.726728107866675</v>
       </c>
     </row>
@@ -2232,28 +2362,33 @@
           <t>eegpt_features/features_sub-026.pt</t>
         </is>
       </c>
-      <c r="J27" t="n">
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-026.pt</t>
+        </is>
+      </c>
+      <c r="K27" t="n">
         <v>0.03317776506211308</v>
       </c>
-      <c r="K27" t="n">
+      <c r="L27" t="n">
         <v>0.04762119072697909</v>
       </c>
-      <c r="L27" t="n">
+      <c r="M27" t="n">
         <v>0.1036645279111386</v>
       </c>
-      <c r="M27" t="n">
+      <c r="N27" t="n">
         <v>0.7950357434882586</v>
       </c>
-      <c r="N27" t="n">
+      <c r="O27" t="n">
         <v>3.14772224304502</v>
       </c>
-      <c r="O27" t="n">
+      <c r="P27" t="n">
         <v>11.58299249242365</v>
       </c>
-      <c r="P27" t="n">
+      <c r="Q27" t="n">
         <v>0.3472103326921244</v>
       </c>
-      <c r="Q27" t="n">
+      <c r="R27" t="n">
         <v>1.927546086603129</v>
       </c>
     </row>
@@ -2299,28 +2434,33 @@
           <t>eegpt_features/features_sub-027.pt</t>
         </is>
       </c>
-      <c r="J28" t="n">
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-027.pt</t>
+        </is>
+      </c>
+      <c r="K28" t="n">
         <v>0.02828043641639512</v>
       </c>
-      <c r="K28" t="n">
+      <c r="L28" t="n">
         <v>0.03494595357188254</v>
       </c>
-      <c r="L28" t="n">
+      <c r="M28" t="n">
         <v>0.1423128472347155</v>
       </c>
-      <c r="M28" t="n">
+      <c r="N28" t="n">
         <v>0.7749130975193266</v>
       </c>
-      <c r="N28" t="n">
+      <c r="O28" t="n">
         <v>5.135041910916232</v>
       </c>
-      <c r="O28" t="n">
+      <c r="P28" t="n">
         <v>14.9340518858637</v>
       </c>
-      <c r="P28" t="n">
+      <c r="Q28" t="n">
         <v>0.3439857724910986</v>
       </c>
-      <c r="Q28" t="n">
+      <c r="R28" t="n">
         <v>1.630054738304451</v>
       </c>
     </row>
@@ -2366,28 +2506,33 @@
           <t>eegpt_features/features_sub-028.pt</t>
         </is>
       </c>
-      <c r="J29" t="n">
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-028.pt</t>
+        </is>
+      </c>
+      <c r="K29" t="n">
         <v>0.03671340279889304</v>
       </c>
-      <c r="K29" t="n">
+      <c r="L29" t="n">
         <v>0.0308118069715708</v>
       </c>
-      <c r="L29" t="n">
+      <c r="M29" t="n">
         <v>0.1175813447720875</v>
       </c>
-      <c r="M29" t="n">
+      <c r="N29" t="n">
         <v>0.7892110981036735</v>
       </c>
-      <c r="N29" t="n">
+      <c r="O29" t="n">
         <v>3.201902403566355</v>
       </c>
-      <c r="O29" t="n">
+      <c r="P29" t="n">
         <v>13.52289529122521</v>
       </c>
-      <c r="P29" t="n">
-        <v>0.3539998328222189</v>
-      </c>
       <c r="Q29" t="n">
+        <v>0.3539998328222188</v>
+      </c>
+      <c r="R29" t="n">
         <v>1.513152461198123</v>
       </c>
     </row>
@@ -2433,28 +2578,33 @@
           <t>eegpt_features/features_sub-029.pt</t>
         </is>
       </c>
-      <c r="J30" t="n">
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-029.pt</t>
+        </is>
+      </c>
+      <c r="K30" t="n">
         <v>0.03294761916527453</v>
       </c>
-      <c r="K30" t="n">
+      <c r="L30" t="n">
         <v>0.0312806113639091</v>
       </c>
-      <c r="L30" t="n">
+      <c r="M30" t="n">
         <v>0.1122072566218513</v>
       </c>
-      <c r="M30" t="n">
+      <c r="N30" t="n">
         <v>0.8019719971850167</v>
       </c>
-      <c r="N30" t="n">
+      <c r="O30" t="n">
         <v>3.431718996007631</v>
       </c>
-      <c r="O30" t="n">
+      <c r="P30" t="n">
         <v>14.65544962303351</v>
       </c>
-      <c r="P30" t="n">
-        <v>0.3481587861785388</v>
-      </c>
       <c r="Q30" t="n">
+        <v>0.3481587861785387</v>
+      </c>
+      <c r="R30" t="n">
         <v>1.534419408671409</v>
       </c>
     </row>
@@ -2500,28 +2650,33 @@
           <t>eegpt_features/features_sub-030.pt</t>
         </is>
       </c>
-      <c r="J31" t="n">
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-030.pt</t>
+        </is>
+      </c>
+      <c r="K31" t="n">
         <v>0.03608115079951266</v>
       </c>
-      <c r="K31" t="n">
+      <c r="L31" t="n">
         <v>0.03076873298102064</v>
       </c>
-      <c r="L31" t="n">
+      <c r="M31" t="n">
         <v>0.1108236889213152</v>
       </c>
-      <c r="M31" t="n">
+      <c r="N31" t="n">
         <v>0.7910643489065554</v>
       </c>
-      <c r="N31" t="n">
+      <c r="O31" t="n">
         <v>3.127938909200892</v>
       </c>
-      <c r="O31" t="n">
+      <c r="P31" t="n">
         <v>13.97009532955569</v>
       </c>
-      <c r="P31" t="n">
+      <c r="Q31" t="n">
         <v>0.2765692640807343</v>
       </c>
-      <c r="Q31" t="n">
+      <c r="R31" t="n">
         <v>1.602879532657042</v>
       </c>
     </row>
@@ -2567,28 +2722,33 @@
           <t>eegpt_features/features_sub-031.pt</t>
         </is>
       </c>
-      <c r="J32" t="n">
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-031.pt</t>
+        </is>
+      </c>
+      <c r="K32" t="n">
         <v>0.04827488240612174</v>
       </c>
-      <c r="K32" t="n">
+      <c r="L32" t="n">
         <v>0.02749658012555351</v>
       </c>
-      <c r="L32" t="n">
+      <c r="M32" t="n">
         <v>0.0858560560200341</v>
       </c>
-      <c r="M32" t="n">
+      <c r="N32" t="n">
         <v>0.8184300322387503</v>
       </c>
-      <c r="N32" t="n">
+      <c r="O32" t="n">
         <v>2.076463164548655</v>
       </c>
-      <c r="O32" t="n">
+      <c r="P32" t="n">
         <v>12.93951452808086</v>
       </c>
-      <c r="P32" t="n">
-        <v>0.3133055110839303</v>
-      </c>
       <c r="Q32" t="n">
+        <v>0.3133055110839302</v>
+      </c>
+      <c r="R32" t="n">
         <v>1.597666309723163</v>
       </c>
     </row>
@@ -2634,28 +2794,33 @@
           <t>eegpt_features/features_sub-032.pt</t>
         </is>
       </c>
-      <c r="J33" t="n">
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-032.pt</t>
+        </is>
+      </c>
+      <c r="K33" t="n">
         <v>0.04355522988546106</v>
       </c>
-      <c r="K33" t="n">
+      <c r="L33" t="n">
         <v>0.04327131357631036</v>
       </c>
-      <c r="L33" t="n">
+      <c r="M33" t="n">
         <v>0.1122794553486255</v>
       </c>
-      <c r="M33" t="n">
+      <c r="N33" t="n">
         <v>0.7724484661543912</v>
       </c>
-      <c r="N33" t="n">
+      <c r="O33" t="n">
         <v>2.636529335444153</v>
       </c>
-      <c r="O33" t="n">
+      <c r="P33" t="n">
         <v>10.42567189442969</v>
       </c>
-      <c r="P33" t="n">
+      <c r="Q33" t="n">
         <v>0.3822144706774575</v>
       </c>
-      <c r="Q33" t="n">
+      <c r="R33" t="n">
         <v>1.762244233212061</v>
       </c>
     </row>
@@ -2701,28 +2866,33 @@
           <t>eegpt_features/features_sub-033.pt</t>
         </is>
       </c>
-      <c r="J34" t="n">
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-033.pt</t>
+        </is>
+      </c>
+      <c r="K34" t="n">
         <v>0.04649542886734834</v>
       </c>
-      <c r="K34" t="n">
+      <c r="L34" t="n">
         <v>0.05458151611152353</v>
       </c>
-      <c r="L34" t="n">
+      <c r="M34" t="n">
         <v>0.09329892959377439</v>
       </c>
-      <c r="M34" t="n">
+      <c r="N34" t="n">
         <v>0.7820131107750266</v>
       </c>
-      <c r="N34" t="n">
+      <c r="O34" t="n">
         <v>2.134231142919547</v>
       </c>
-      <c r="O34" t="n">
+      <c r="P34" t="n">
         <v>9.055141729500102</v>
       </c>
-      <c r="P34" t="n">
+      <c r="Q34" t="n">
         <v>0.2878619953812484</v>
       </c>
-      <c r="Q34" t="n">
+      <c r="R34" t="n">
         <v>1.666875342394489</v>
       </c>
     </row>
@@ -2768,28 +2938,33 @@
           <t>eegpt_features/features_sub-034.pt</t>
         </is>
       </c>
-      <c r="J35" t="n">
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-034.pt</t>
+        </is>
+      </c>
+      <c r="K35" t="n">
         <v>0.02949036571175536</v>
       </c>
-      <c r="K35" t="n">
+      <c r="L35" t="n">
         <v>0.02959264641360278</v>
       </c>
-      <c r="L35" t="n">
+      <c r="M35" t="n">
         <v>0.09877156876394308</v>
       </c>
-      <c r="M35" t="n">
+      <c r="N35" t="n">
         <v>0.8235206849690084</v>
       </c>
-      <c r="N35" t="n">
+      <c r="O35" t="n">
         <v>3.374824857178436</v>
       </c>
-      <c r="O35" t="n">
+      <c r="P35" t="n">
         <v>15.79412574499994</v>
       </c>
-      <c r="P35" t="n">
+      <c r="Q35" t="n">
         <v>0.3995510660080305</v>
       </c>
-      <c r="Q35" t="n">
+      <c r="R35" t="n">
         <v>1.426935593156887</v>
       </c>
     </row>
@@ -2835,28 +3010,33 @@
           <t>eegpt_features/features_sub-035.pt</t>
         </is>
       </c>
-      <c r="J36" t="n">
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-035.pt</t>
+        </is>
+      </c>
+      <c r="K36" t="n">
         <v>0.03539753656490721</v>
       </c>
-      <c r="K36" t="n">
+      <c r="L36" t="n">
         <v>0.03224110175840138</v>
       </c>
-      <c r="L36" t="n">
+      <c r="M36" t="n">
         <v>0.09956031551266475</v>
       </c>
-      <c r="M36" t="n">
+      <c r="N36" t="n">
         <v>0.8086209181228118</v>
       </c>
-      <c r="N36" t="n">
+      <c r="O36" t="n">
         <v>2.83201479405633</v>
       </c>
-      <c r="O36" t="n">
+      <c r="P36" t="n">
         <v>13.65682234641099</v>
       </c>
-      <c r="P36" t="n">
+      <c r="Q36" t="n">
         <v>0.3640743717020201</v>
       </c>
-      <c r="Q36" t="n">
+      <c r="R36" t="n">
         <v>1.513298778626837</v>
       </c>
     </row>
@@ -2902,28 +3082,33 @@
           <t>eegpt_features/features_sub-036.pt</t>
         </is>
       </c>
-      <c r="J37" t="n">
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-036.pt</t>
+        </is>
+      </c>
+      <c r="K37" t="n">
         <v>0.08263173545211451</v>
       </c>
-      <c r="K37" t="n">
+      <c r="L37" t="n">
         <v>0.07521227928840213</v>
       </c>
-      <c r="L37" t="n">
+      <c r="M37" t="n">
         <v>0.08697933745598617</v>
       </c>
-      <c r="M37" t="n">
+      <c r="N37" t="n">
         <v>0.7177029427320281</v>
       </c>
-      <c r="N37" t="n">
+      <c r="O37" t="n">
         <v>1.100695964139083</v>
       </c>
-      <c r="O37" t="n">
+      <c r="P37" t="n">
         <v>5.233560200407738</v>
       </c>
-      <c r="P37" t="n">
+      <c r="Q37" t="n">
         <v>0.2488973337392034</v>
       </c>
-      <c r="Q37" t="n">
+      <c r="R37" t="n">
         <v>1.838486242471856</v>
       </c>
     </row>
@@ -2969,28 +3154,33 @@
           <t>eegpt_features/features_sub-037.pt</t>
         </is>
       </c>
-      <c r="J38" t="n">
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-037.pt</t>
+        </is>
+      </c>
+      <c r="K38" t="n">
         <v>0.1039798606515489</v>
       </c>
-      <c r="K38" t="n">
+      <c r="L38" t="n">
         <v>0.03148155974255468</v>
       </c>
-      <c r="L38" t="n">
+      <c r="M38" t="n">
         <v>0.08049206327227053</v>
       </c>
-      <c r="M38" t="n">
+      <c r="N38" t="n">
         <v>0.7532093833404663</v>
       </c>
-      <c r="N38" t="n">
+      <c r="O38" t="n">
         <v>1.135075212301661</v>
       </c>
-      <c r="O38" t="n">
+      <c r="P38" t="n">
         <v>7.813967181366159</v>
       </c>
-      <c r="P38" t="n">
+      <c r="Q38" t="n">
         <v>0.329712820078321</v>
       </c>
-      <c r="Q38" t="n">
+      <c r="R38" t="n">
         <v>1.581531180338038</v>
       </c>
     </row>
@@ -3036,28 +3226,33 @@
           <t>eegpt_features/features_sub-038.pt</t>
         </is>
       </c>
-      <c r="J39" t="n">
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-038.pt</t>
+        </is>
+      </c>
+      <c r="K39" t="n">
         <v>0.05166088405299617</v>
       </c>
-      <c r="K39" t="n">
+      <c r="L39" t="n">
         <v>0.04477894353217218</v>
       </c>
-      <c r="L39" t="n">
+      <c r="M39" t="n">
         <v>0.09667257346991558</v>
       </c>
-      <c r="M39" t="n">
+      <c r="N39" t="n">
         <v>0.7875474082255937</v>
       </c>
-      <c r="N39" t="n">
+      <c r="O39" t="n">
         <v>2.143542550114836</v>
       </c>
-      <c r="O39" t="n">
+      <c r="P39" t="n">
         <v>9.716896003734917</v>
       </c>
-      <c r="P39" t="n">
-        <v>0.3478255991504391</v>
-      </c>
       <c r="Q39" t="n">
+        <v>0.3478255991504392</v>
+      </c>
+      <c r="R39" t="n">
         <v>1.570600036297451</v>
       </c>
     </row>
@@ -3103,28 +3298,33 @@
           <t>eegpt_features/features_sub-039.pt</t>
         </is>
       </c>
-      <c r="J40" t="n">
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-039.pt</t>
+        </is>
+      </c>
+      <c r="K40" t="n">
         <v>0.1575382517832842</v>
       </c>
-      <c r="K40" t="n">
+      <c r="L40" t="n">
         <v>0.04360816311209056</v>
       </c>
-      <c r="L40" t="n">
+      <c r="M40" t="n">
         <v>0.0804681372474757</v>
       </c>
-      <c r="M40" t="n">
+      <c r="N40" t="n">
         <v>0.6894950856840188</v>
       </c>
-      <c r="N40" t="n">
+      <c r="O40" t="n">
         <v>0.618386609221897</v>
       </c>
-      <c r="O40" t="n">
+      <c r="P40" t="n">
         <v>4.354684095598305</v>
       </c>
-      <c r="P40" t="n">
+      <c r="Q40" t="n">
         <v>0.2981288299889995</v>
       </c>
-      <c r="Q40" t="n">
+      <c r="R40" t="n">
         <v>1.813254983363934</v>
       </c>
     </row>
@@ -3170,28 +3370,33 @@
           <t>eegpt_features/features_sub-040.pt</t>
         </is>
       </c>
-      <c r="J41" t="n">
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-040.pt</t>
+        </is>
+      </c>
+      <c r="K41" t="n">
         <v>0.07424603316966162</v>
       </c>
-      <c r="K41" t="n">
+      <c r="L41" t="n">
         <v>0.03637445177925219</v>
       </c>
-      <c r="L41" t="n">
+      <c r="M41" t="n">
         <v>0.08083781677751704</v>
       </c>
-      <c r="M41" t="n">
+      <c r="N41" t="n">
         <v>0.7889258843110887</v>
       </c>
-      <c r="N41" t="n">
+      <c r="O41" t="n">
         <v>1.406945732210052</v>
       </c>
-      <c r="O41" t="n">
+      <c r="P41" t="n">
         <v>9.186311343934021</v>
       </c>
-      <c r="P41" t="n">
+      <c r="Q41" t="n">
         <v>0.2840169940868846</v>
       </c>
-      <c r="Q41" t="n">
+      <c r="R41" t="n">
         <v>1.572829976061636</v>
       </c>
     </row>
@@ -3237,28 +3442,33 @@
           <t>eegpt_features/features_sub-041.pt</t>
         </is>
       </c>
-      <c r="J42" t="n">
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-041.pt</t>
+        </is>
+      </c>
+      <c r="K42" t="n">
         <v>0.0359819940714077</v>
       </c>
-      <c r="K42" t="n">
+      <c r="L42" t="n">
         <v>0.04443219149370312</v>
       </c>
-      <c r="L42" t="n">
+      <c r="M42" t="n">
         <v>0.08332028026283154</v>
       </c>
-      <c r="M42" t="n">
+      <c r="N42" t="n">
         <v>0.8185980464677238</v>
       </c>
-      <c r="N42" t="n">
+      <c r="O42" t="n">
         <v>2.456271420015434</v>
       </c>
-      <c r="O42" t="n">
+      <c r="P42" t="n">
         <v>12.21439676640319</v>
       </c>
-      <c r="P42" t="n">
+      <c r="Q42" t="n">
         <v>0.3390838501411498</v>
       </c>
-      <c r="Q42" t="n">
+      <c r="R42" t="n">
         <v>1.588590040583802</v>
       </c>
     </row>
@@ -3304,28 +3514,33 @@
           <t>eegpt_features/features_sub-042.pt</t>
         </is>
       </c>
-      <c r="J43" t="n">
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-042.pt</t>
+        </is>
+      </c>
+      <c r="K43" t="n">
         <v>0.06783643085015116</v>
       </c>
-      <c r="K43" t="n">
+      <c r="L43" t="n">
         <v>0.03948267343873091</v>
       </c>
-      <c r="L43" t="n">
+      <c r="M43" t="n">
         <v>0.082480774181438</v>
       </c>
-      <c r="M43" t="n">
+      <c r="N43" t="n">
         <v>0.7910332183681493</v>
       </c>
-      <c r="N43" t="n">
+      <c r="O43" t="n">
         <v>1.587501105678099</v>
       </c>
-      <c r="O43" t="n">
+      <c r="P43" t="n">
         <v>9.874547196602496</v>
       </c>
-      <c r="P43" t="n">
+      <c r="Q43" t="n">
         <v>0.2826344206656418</v>
       </c>
-      <c r="Q43" t="n">
+      <c r="R43" t="n">
         <v>1.55739139677244</v>
       </c>
     </row>
@@ -3371,28 +3586,33 @@
           <t>eegpt_features/features_sub-043.pt</t>
         </is>
       </c>
-      <c r="J44" t="n">
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-043.pt</t>
+        </is>
+      </c>
+      <c r="K44" t="n">
         <v>0.03211927293519624</v>
       </c>
-      <c r="K44" t="n">
+      <c r="L44" t="n">
         <v>0.03042848441314668</v>
       </c>
-      <c r="L44" t="n">
+      <c r="M44" t="n">
         <v>0.0870215820140494</v>
       </c>
-      <c r="M44" t="n">
+      <c r="N44" t="n">
         <v>0.8335999629812284</v>
       </c>
-      <c r="N44" t="n">
+      <c r="O44" t="n">
         <v>2.761228584935738</v>
       </c>
-      <c r="O44" t="n">
+      <c r="P44" t="n">
         <v>15.06871125778666</v>
       </c>
-      <c r="P44" t="n">
+      <c r="Q44" t="n">
         <v>0.3685436122748043</v>
       </c>
-      <c r="Q44" t="n">
+      <c r="R44" t="n">
         <v>1.446049288096347</v>
       </c>
     </row>
@@ -3438,28 +3658,33 @@
           <t>eegpt_features/features_sub-044.pt</t>
         </is>
       </c>
-      <c r="J45" t="n">
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-044.pt</t>
+        </is>
+      </c>
+      <c r="K45" t="n">
         <v>0.08304704984061491</v>
       </c>
-      <c r="K45" t="n">
+      <c r="L45" t="n">
         <v>0.03495697993746733</v>
       </c>
-      <c r="L45" t="n">
+      <c r="M45" t="n">
         <v>0.0813397739814551</v>
       </c>
-      <c r="M45" t="n">
+      <c r="N45" t="n">
         <v>0.7817406399414309</v>
       </c>
-      <c r="N45" t="n">
+      <c r="O45" t="n">
         <v>1.282728232273807</v>
       </c>
-      <c r="O45" t="n">
+      <c r="P45" t="n">
         <v>8.703636935076485</v>
       </c>
-      <c r="P45" t="n">
+      <c r="Q45" t="n">
         <v>0.2984988458692158</v>
       </c>
-      <c r="Q45" t="n">
+      <c r="R45" t="n">
         <v>1.59181384912629</v>
       </c>
     </row>
@@ -3505,28 +3730,33 @@
           <t>eegpt_features/features_sub-045.pt</t>
         </is>
       </c>
-      <c r="J46" t="n">
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-045.pt</t>
+        </is>
+      </c>
+      <c r="K46" t="n">
         <v>0.03688695762457282</v>
       </c>
-      <c r="K46" t="n">
+      <c r="L46" t="n">
         <v>0.03328587215591617</v>
       </c>
-      <c r="L46" t="n">
+      <c r="M46" t="n">
         <v>0.09403306702375933</v>
       </c>
-      <c r="M46" t="n">
+      <c r="N46" t="n">
         <v>0.8147966641988854</v>
       </c>
-      <c r="N46" t="n">
+      <c r="O46" t="n">
         <v>2.635621607663999</v>
       </c>
-      <c r="O46" t="n">
+      <c r="P46" t="n">
         <v>13.39665546097676</v>
       </c>
-      <c r="P46" t="n">
-        <v>0.3346654573361177</v>
-      </c>
       <c r="Q46" t="n">
+        <v>0.3346654573361178</v>
+      </c>
+      <c r="R46" t="n">
         <v>1.496733957897642</v>
       </c>
     </row>
@@ -3572,28 +3802,33 @@
           <t>eegpt_features/features_sub-046.pt</t>
         </is>
       </c>
-      <c r="J47" t="n">
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-046.pt</t>
+        </is>
+      </c>
+      <c r="K47" t="n">
         <v>0.09622658913210423</v>
       </c>
-      <c r="K47" t="n">
+      <c r="L47" t="n">
         <v>0.06779561694525749</v>
       </c>
-      <c r="L47" t="n">
+      <c r="M47" t="n">
         <v>0.1043138478835941</v>
       </c>
-      <c r="M47" t="n">
+      <c r="N47" t="n">
         <v>0.6988581165708065</v>
       </c>
-      <c r="N47" t="n">
+      <c r="O47" t="n">
         <v>1.213154175938766</v>
       </c>
-      <c r="O47" t="n">
+      <c r="P47" t="n">
         <v>5.211093184461276</v>
       </c>
-      <c r="P47" t="n">
-        <v>0.2554932281380665</v>
-      </c>
       <c r="Q47" t="n">
+        <v>0.2554932281380664</v>
+      </c>
+      <c r="R47" t="n">
         <v>1.8201489466769</v>
       </c>
     </row>
@@ -3639,28 +3874,33 @@
           <t>eegpt_features/features_sub-047.pt</t>
         </is>
       </c>
-      <c r="J48" t="n">
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-047.pt</t>
+        </is>
+      </c>
+      <c r="K48" t="n">
         <v>0.07116895708288319</v>
       </c>
-      <c r="K48" t="n">
+      <c r="L48" t="n">
         <v>0.03575747528388498</v>
       </c>
-      <c r="L48" t="n">
+      <c r="M48" t="n">
         <v>0.08599633185640909</v>
       </c>
-      <c r="M48" t="n">
+      <c r="N48" t="n">
         <v>0.7861385655160082</v>
       </c>
-      <c r="N48" t="n">
+      <c r="O48" t="n">
         <v>1.438431063264973</v>
       </c>
-      <c r="O48" t="n">
+      <c r="P48" t="n">
         <v>9.203185225962057</v>
       </c>
-      <c r="P48" t="n">
+      <c r="Q48" t="n">
         <v>0.2723195983747117</v>
       </c>
-      <c r="Q48" t="n">
+      <c r="R48" t="n">
         <v>1.597050373842684</v>
       </c>
     </row>
@@ -3706,28 +3946,33 @@
           <t>eegpt_features/features_sub-048.pt</t>
         </is>
       </c>
-      <c r="J49" t="n">
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-048.pt</t>
+        </is>
+      </c>
+      <c r="K49" t="n">
         <v>0.06471009412679596</v>
       </c>
-      <c r="K49" t="n">
+      <c r="L49" t="n">
         <v>0.03586735655454534</v>
       </c>
-      <c r="L49" t="n">
+      <c r="M49" t="n">
         <v>0.08242613457346259</v>
       </c>
-      <c r="M49" t="n">
+      <c r="N49" t="n">
         <v>0.7985712399213414</v>
       </c>
-      <c r="N49" t="n">
+      <c r="O49" t="n">
         <v>1.743597892820584</v>
       </c>
-      <c r="O49" t="n">
+      <c r="P49" t="n">
         <v>10.57977752970212</v>
       </c>
-      <c r="P49" t="n">
-        <v>0.2940379516429639</v>
-      </c>
       <c r="Q49" t="n">
+        <v>0.294037951642964</v>
+      </c>
+      <c r="R49" t="n">
         <v>1.639260881193106</v>
       </c>
     </row>
@@ -3773,28 +4018,33 @@
           <t>eegpt_features/features_sub-049.pt</t>
         </is>
       </c>
-      <c r="J50" t="n">
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-049.pt</t>
+        </is>
+      </c>
+      <c r="K50" t="n">
         <v>0.07878520627051741</v>
       </c>
-      <c r="K50" t="n">
+      <c r="L50" t="n">
         <v>0.04145163106753308</v>
       </c>
-      <c r="L50" t="n">
+      <c r="M50" t="n">
         <v>0.08534754071169966</v>
       </c>
-      <c r="M50" t="n">
+      <c r="N50" t="n">
         <v>0.7751548740401066</v>
       </c>
-      <c r="N50" t="n">
+      <c r="O50" t="n">
         <v>1.71828504434369</v>
       </c>
-      <c r="O50" t="n">
+      <c r="P50" t="n">
         <v>9.668909495459374</v>
       </c>
-      <c r="P50" t="n">
+      <c r="Q50" t="n">
         <v>0.2984152125750761</v>
       </c>
-      <c r="Q50" t="n">
+      <c r="R50" t="n">
         <v>1.619677665591375</v>
       </c>
     </row>
@@ -3840,28 +4090,33 @@
           <t>eegpt_features/features_sub-050.pt</t>
         </is>
       </c>
-      <c r="J51" t="n">
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-050.pt</t>
+        </is>
+      </c>
+      <c r="K51" t="n">
         <v>0.05422881718805344</v>
       </c>
-      <c r="K51" t="n">
+      <c r="L51" t="n">
         <v>0.03555201253916864</v>
       </c>
-      <c r="L51" t="n">
+      <c r="M51" t="n">
         <v>0.08615589601194154</v>
       </c>
-      <c r="M51" t="n">
+      <c r="N51" t="n">
         <v>0.7929076613259645</v>
       </c>
-      <c r="N51" t="n">
+      <c r="O51" t="n">
         <v>1.906009725277412</v>
       </c>
-      <c r="O51" t="n">
+      <c r="P51" t="n">
         <v>10.86407856848967</v>
       </c>
-      <c r="P51" t="n">
+      <c r="Q51" t="n">
         <v>0.3125247255848122</v>
       </c>
-      <c r="Q51" t="n">
+      <c r="R51" t="n">
         <v>1.576621121298419</v>
       </c>
     </row>
@@ -3907,28 +4162,33 @@
           <t>eegpt_features/features_sub-051.pt</t>
         </is>
       </c>
-      <c r="J52" t="n">
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-051.pt</t>
+        </is>
+      </c>
+      <c r="K52" t="n">
         <v>0.04456350769550512</v>
       </c>
-      <c r="K52" t="n">
+      <c r="L52" t="n">
         <v>0.03397485162751562</v>
       </c>
-      <c r="L52" t="n">
+      <c r="M52" t="n">
         <v>0.0821535238486351</v>
       </c>
-      <c r="M52" t="n">
+      <c r="N52" t="n">
         <v>0.8215251398130149</v>
       </c>
-      <c r="N52" t="n">
+      <c r="O52" t="n">
         <v>1.974371502583209</v>
       </c>
-      <c r="O52" t="n">
+      <c r="P52" t="n">
         <v>12.1154753882443</v>
       </c>
-      <c r="P52" t="n">
+      <c r="Q52" t="n">
         <v>0.3112999855816281</v>
       </c>
-      <c r="Q52" t="n">
+      <c r="R52" t="n">
         <v>1.490731668510016</v>
       </c>
     </row>
@@ -3974,28 +4234,33 @@
           <t>eegpt_features/features_sub-052.pt</t>
         </is>
       </c>
-      <c r="J53" t="n">
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-052.pt</t>
+        </is>
+      </c>
+      <c r="K53" t="n">
         <v>0.05534494600450018</v>
       </c>
-      <c r="K53" t="n">
+      <c r="L53" t="n">
         <v>0.04647466774887992</v>
       </c>
-      <c r="L53" t="n">
+      <c r="M53" t="n">
         <v>0.08796582349711299</v>
       </c>
-      <c r="M53" t="n">
+      <c r="N53" t="n">
         <v>0.7890716378019749</v>
       </c>
-      <c r="N53" t="n">
+      <c r="O53" t="n">
         <v>1.716759307206788</v>
       </c>
-      <c r="O53" t="n">
+      <c r="P53" t="n">
         <v>8.999671118112278</v>
       </c>
-      <c r="P53" t="n">
+      <c r="Q53" t="n">
         <v>0.2826343537388473</v>
       </c>
-      <c r="Q53" t="n">
+      <c r="R53" t="n">
         <v>1.636213392560241</v>
       </c>
     </row>
@@ -4041,28 +4306,33 @@
           <t>eegpt_features/features_sub-053.pt</t>
         </is>
       </c>
-      <c r="J54" t="n">
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-053.pt</t>
+        </is>
+      </c>
+      <c r="K54" t="n">
         <v>0.08796207048943568</v>
       </c>
-      <c r="K54" t="n">
+      <c r="L54" t="n">
         <v>0.04324482412819373</v>
       </c>
-      <c r="L54" t="n">
+      <c r="M54" t="n">
         <v>0.08142279240438899</v>
       </c>
-      <c r="M54" t="n">
+      <c r="N54" t="n">
         <v>0.7516243173353827</v>
       </c>
-      <c r="N54" t="n">
+      <c r="O54" t="n">
         <v>1.21968836356075</v>
       </c>
-      <c r="O54" t="n">
+      <c r="P54" t="n">
         <v>7.872022745300694</v>
       </c>
-      <c r="P54" t="n">
+      <c r="Q54" t="n">
         <v>0.2746734690292134</v>
       </c>
-      <c r="Q54" t="n">
+      <c r="R54" t="n">
         <v>1.70872624161361</v>
       </c>
     </row>
@@ -4108,28 +4378,33 @@
           <t>eegpt_features/features_sub-054.pt</t>
         </is>
       </c>
-      <c r="J55" t="n">
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-054.pt</t>
+        </is>
+      </c>
+      <c r="K55" t="n">
         <v>0.1038313680217803</v>
       </c>
-      <c r="K55" t="n">
+      <c r="L55" t="n">
         <v>0.04241670891735033</v>
       </c>
-      <c r="L55" t="n">
+      <c r="M55" t="n">
         <v>0.08576732026561446</v>
       </c>
-      <c r="M55" t="n">
+      <c r="N55" t="n">
         <v>0.7408571435359534</v>
       </c>
-      <c r="N55" t="n">
+      <c r="O55" t="n">
         <v>1.150889038527123</v>
       </c>
-      <c r="O55" t="n">
+      <c r="P55" t="n">
         <v>7.078198777344476</v>
       </c>
-      <c r="P55" t="n">
-        <v>0.2672440421240836</v>
-      </c>
       <c r="Q55" t="n">
+        <v>0.2672440421240837</v>
+      </c>
+      <c r="R55" t="n">
         <v>1.684213118365308</v>
       </c>
     </row>
@@ -4175,28 +4450,33 @@
           <t>eegpt_features/features_sub-055.pt</t>
         </is>
       </c>
-      <c r="J56" t="n">
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-055.pt</t>
+        </is>
+      </c>
+      <c r="K56" t="n">
         <v>0.05366586315071798</v>
       </c>
-      <c r="K56" t="n">
+      <c r="L56" t="n">
         <v>0.0626787929980461</v>
       </c>
-      <c r="L56" t="n">
+      <c r="M56" t="n">
         <v>0.08843368965145321</v>
       </c>
-      <c r="M56" t="n">
+      <c r="N56" t="n">
         <v>0.771130135647847</v>
       </c>
-      <c r="N56" t="n">
+      <c r="O56" t="n">
         <v>1.964967355376197</v>
       </c>
-      <c r="O56" t="n">
+      <c r="P56" t="n">
         <v>8.025711364069794</v>
       </c>
-      <c r="P56" t="n">
-        <v>0.3131886253410081</v>
-      </c>
       <c r="Q56" t="n">
+        <v>0.3131886253410079</v>
+      </c>
+      <c r="R56" t="n">
         <v>1.674772937927566</v>
       </c>
     </row>
@@ -4242,28 +4522,33 @@
           <t>eegpt_features/features_sub-056.pt</t>
         </is>
       </c>
-      <c r="J57" t="n">
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-056.pt</t>
+        </is>
+      </c>
+      <c r="K57" t="n">
         <v>0.1235538025056778</v>
       </c>
-      <c r="K57" t="n">
+      <c r="L57" t="n">
         <v>0.04425195502748489</v>
       </c>
-      <c r="L57" t="n">
+      <c r="M57" t="n">
         <v>0.1114003458822174</v>
       </c>
-      <c r="M57" t="n">
+      <c r="N57" t="n">
         <v>0.6918360201392223</v>
       </c>
-      <c r="N57" t="n">
+      <c r="O57" t="n">
         <v>1.079223451151476</v>
       </c>
-      <c r="O57" t="n">
+      <c r="P57" t="n">
         <v>5.343137565642841</v>
       </c>
-      <c r="P57" t="n">
-        <v>0.3482854282981004</v>
-      </c>
       <c r="Q57" t="n">
+        <v>0.3482854282981003</v>
+      </c>
+      <c r="R57" t="n">
         <v>2.275114752292621</v>
       </c>
     </row>
@@ -4309,28 +4594,33 @@
           <t>eegpt_features/features_sub-057.pt</t>
         </is>
       </c>
-      <c r="J58" t="n">
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-057.pt</t>
+        </is>
+      </c>
+      <c r="K58" t="n">
         <v>0.06444228831401896</v>
       </c>
-      <c r="K58" t="n">
+      <c r="L58" t="n">
         <v>0.03913297741751334</v>
       </c>
-      <c r="L58" t="n">
+      <c r="M58" t="n">
         <v>0.08429695192434067</v>
       </c>
-      <c r="M58" t="n">
+      <c r="N58" t="n">
         <v>0.791909681396805</v>
       </c>
-      <c r="N58" t="n">
+      <c r="O58" t="n">
         <v>1.691507152405973</v>
       </c>
-      <c r="O58" t="n">
+      <c r="P58" t="n">
         <v>9.871700419208828</v>
       </c>
-      <c r="P58" t="n">
-        <v>0.3039355915375853</v>
-      </c>
       <c r="Q58" t="n">
+        <v>0.3039355915375854</v>
+      </c>
+      <c r="R58" t="n">
         <v>1.554099887426237</v>
       </c>
     </row>
@@ -4376,28 +4666,33 @@
           <t>eegpt_features/features_sub-058.pt</t>
         </is>
       </c>
-      <c r="J59" t="n">
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-058.pt</t>
+        </is>
+      </c>
+      <c r="K59" t="n">
         <v>0.07255057428853738</v>
       </c>
-      <c r="K59" t="n">
+      <c r="L59" t="n">
         <v>0.04984200548037316</v>
       </c>
-      <c r="L59" t="n">
+      <c r="M59" t="n">
         <v>0.08207528333720837</v>
       </c>
-      <c r="M59" t="n">
+      <c r="N59" t="n">
         <v>0.7747841533174221</v>
       </c>
-      <c r="N59" t="n">
+      <c r="O59" t="n">
         <v>1.351938067739232</v>
       </c>
-      <c r="O59" t="n">
+      <c r="P59" t="n">
         <v>7.806527799466269</v>
       </c>
-      <c r="P59" t="n">
+      <c r="Q59" t="n">
         <v>0.2815374057676726</v>
       </c>
-      <c r="Q59" t="n">
+      <c r="R59" t="n">
         <v>1.654270698046675</v>
       </c>
     </row>
@@ -4443,28 +4738,33 @@
           <t>eegpt_features/features_sub-059.pt</t>
         </is>
       </c>
-      <c r="J60" t="n">
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-059.pt</t>
+        </is>
+      </c>
+      <c r="K60" t="n">
         <v>0.03081800332792686</v>
       </c>
-      <c r="K60" t="n">
+      <c r="L60" t="n">
         <v>0.03358337426425888</v>
       </c>
-      <c r="L60" t="n">
+      <c r="M60" t="n">
         <v>0.08586261538697501</v>
       </c>
-      <c r="M60" t="n">
+      <c r="N60" t="n">
         <v>0.8322588404151483</v>
       </c>
-      <c r="N60" t="n">
+      <c r="O60" t="n">
         <v>2.813158286189048</v>
       </c>
-      <c r="O60" t="n">
+      <c r="P60" t="n">
         <v>14.53844198805961</v>
       </c>
-      <c r="P60" t="n">
-        <v>0.3700622873869278</v>
-      </c>
       <c r="Q60" t="n">
+        <v>0.370062287386928</v>
+      </c>
+      <c r="R60" t="n">
         <v>1.436827535766982</v>
       </c>
     </row>
@@ -4510,28 +4810,33 @@
           <t>eegpt_features/features_sub-060.pt</t>
         </is>
       </c>
-      <c r="J61" t="n">
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-060.pt</t>
+        </is>
+      </c>
+      <c r="K61" t="n">
         <v>0.02947098390539975</v>
       </c>
-      <c r="K61" t="n">
+      <c r="L61" t="n">
         <v>0.03986205066612204</v>
       </c>
-      <c r="L61" t="n">
+      <c r="M61" t="n">
         <v>0.08719111839730365</v>
       </c>
-      <c r="M61" t="n">
+      <c r="N61" t="n">
         <v>0.8255112291994532</v>
       </c>
-      <c r="N61" t="n">
+      <c r="O61" t="n">
         <v>2.997301882365906</v>
       </c>
-      <c r="O61" t="n">
+      <c r="P61" t="n">
         <v>13.55291460008928</v>
       </c>
-      <c r="P61" t="n">
+      <c r="Q61" t="n">
         <v>0.3973900393901326</v>
       </c>
-      <c r="Q61" t="n">
+      <c r="R61" t="n">
         <v>1.464326189145709</v>
       </c>
     </row>
@@ -4577,28 +4882,33 @@
           <t>eegpt_features/features_sub-061.pt</t>
         </is>
       </c>
-      <c r="J62" t="n">
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-061.pt</t>
+        </is>
+      </c>
+      <c r="K62" t="n">
         <v>0.03645803904409222</v>
       </c>
-      <c r="K62" t="n">
+      <c r="L62" t="n">
         <v>0.0272829048639637</v>
       </c>
-      <c r="L62" t="n">
+      <c r="M62" t="n">
         <v>0.08402675503122846</v>
       </c>
-      <c r="M62" t="n">
+      <c r="N62" t="n">
         <v>0.8355702465298528</v>
       </c>
-      <c r="N62" t="n">
+      <c r="O62" t="n">
         <v>2.486725603808816</v>
       </c>
-      <c r="O62" t="n">
+      <c r="P62" t="n">
         <v>15.00802739752978</v>
       </c>
-      <c r="P62" t="n">
-        <v>0.3403600680401337</v>
-      </c>
       <c r="Q62" t="n">
+        <v>0.340360068040134</v>
+      </c>
+      <c r="R62" t="n">
         <v>1.498642141026646</v>
       </c>
     </row>
@@ -4644,28 +4954,33 @@
           <t>eegpt_features/features_sub-062.pt</t>
         </is>
       </c>
-      <c r="J63" t="n">
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-062.pt</t>
+        </is>
+      </c>
+      <c r="K63" t="n">
         <v>0.1135962197471351</v>
       </c>
-      <c r="K63" t="n">
+      <c r="L63" t="n">
         <v>0.0349432828862697</v>
       </c>
-      <c r="L63" t="n">
+      <c r="M63" t="n">
         <v>0.08588835589385602</v>
       </c>
-      <c r="M63" t="n">
+      <c r="N63" t="n">
         <v>0.7450891650955275</v>
       </c>
-      <c r="N63" t="n">
+      <c r="O63" t="n">
         <v>1.200808543296274</v>
       </c>
-      <c r="O63" t="n">
+      <c r="P63" t="n">
         <v>7.44002078487558</v>
       </c>
-      <c r="P63" t="n">
+      <c r="Q63" t="n">
         <v>0.3067347614222961</v>
       </c>
-      <c r="Q63" t="n">
+      <c r="R63" t="n">
         <v>1.606037143814291</v>
       </c>
     </row>
@@ -4711,28 +5026,33 @@
           <t>eegpt_features/features_sub-063.pt</t>
         </is>
       </c>
-      <c r="J64" t="n">
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-063.pt</t>
+        </is>
+      </c>
+      <c r="K64" t="n">
         <v>0.04082591527902577</v>
       </c>
-      <c r="K64" t="n">
+      <c r="L64" t="n">
         <v>0.03842617030003326</v>
       </c>
-      <c r="L64" t="n">
+      <c r="M64" t="n">
         <v>0.09786932588023275</v>
       </c>
-      <c r="M64" t="n">
+      <c r="N64" t="n">
         <v>0.8035484364663205</v>
       </c>
-      <c r="N64" t="n">
+      <c r="O64" t="n">
         <v>2.522465049858871</v>
       </c>
-      <c r="O64" t="n">
+      <c r="P64" t="n">
         <v>11.75978076032396</v>
       </c>
-      <c r="P64" t="n">
+      <c r="Q64" t="n">
         <v>0.35237242521585</v>
       </c>
-      <c r="Q64" t="n">
+      <c r="R64" t="n">
         <v>1.521717483183683</v>
       </c>
     </row>
@@ -4778,28 +5098,33 @@
           <t>eegpt_features/features_sub-064.pt</t>
         </is>
       </c>
-      <c r="J65" t="n">
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-064.pt</t>
+        </is>
+      </c>
+      <c r="K65" t="n">
         <v>0.1742157978923472</v>
       </c>
-      <c r="K65" t="n">
+      <c r="L65" t="n">
         <v>0.05064184183041267</v>
       </c>
-      <c r="L65" t="n">
+      <c r="M65" t="n">
         <v>0.07226151088634702</v>
       </c>
-      <c r="M65" t="n">
+      <c r="N65" t="n">
         <v>0.6775793361451666</v>
       </c>
-      <c r="N65" t="n">
+      <c r="O65" t="n">
         <v>0.5709713328037825</v>
       </c>
-      <c r="O65" t="n">
+      <c r="P65" t="n">
         <v>4.184699767625244</v>
       </c>
-      <c r="P65" t="n">
-        <v>0.2562471113334038</v>
-      </c>
       <c r="Q65" t="n">
+        <v>0.2562471113334039</v>
+      </c>
+      <c r="R65" t="n">
         <v>1.807481225079709</v>
       </c>
     </row>
@@ -4845,28 +5170,33 @@
           <t>eegpt_features/features_sub-065.pt</t>
         </is>
       </c>
-      <c r="J66" t="n">
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-065.pt</t>
+        </is>
+      </c>
+      <c r="K66" t="n">
         <v>0.03696614874867402</v>
       </c>
-      <c r="K66" t="n">
+      <c r="L66" t="n">
         <v>0.03482522066133191</v>
       </c>
-      <c r="L66" t="n">
+      <c r="M66" t="n">
         <v>0.0807494185219642</v>
       </c>
-      <c r="M66" t="n">
+      <c r="N66" t="n">
         <v>0.8301571349250417</v>
       </c>
-      <c r="N66" t="n">
+      <c r="O66" t="n">
         <v>2.50064489857262</v>
       </c>
-      <c r="O66" t="n">
+      <c r="P66" t="n">
         <v>13.65895134313799</v>
       </c>
-      <c r="P66" t="n">
+      <c r="Q66" t="n">
         <v>0.3540412838848526</v>
       </c>
-      <c r="Q66" t="n">
+      <c r="R66" t="n">
         <v>1.485236590519807</v>
       </c>
     </row>
@@ -4912,28 +5242,33 @@
           <t>eegpt_features/features_sub-066.pt</t>
         </is>
       </c>
-      <c r="J67" t="n">
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-066.pt</t>
+        </is>
+      </c>
+      <c r="K67" t="n">
         <v>0.04907626931434481</v>
       </c>
-      <c r="K67" t="n">
+      <c r="L67" t="n">
         <v>0.02952592129111201</v>
       </c>
-      <c r="L67" t="n">
+      <c r="M67" t="n">
         <v>0.09978061462392718</v>
       </c>
-      <c r="M67" t="n">
+      <c r="N67" t="n">
         <v>0.7841852853367722</v>
       </c>
-      <c r="N67" t="n">
+      <c r="O67" t="n">
         <v>2.067466826052398</v>
       </c>
-      <c r="O67" t="n">
+      <c r="P67" t="n">
         <v>11.38694135920838</v>
       </c>
-      <c r="P67" t="n">
+      <c r="Q67" t="n">
         <v>0.2909411630482368</v>
       </c>
-      <c r="Q67" t="n">
+      <c r="R67" t="n">
         <v>1.607083986326283</v>
       </c>
     </row>
@@ -4979,28 +5314,33 @@
           <t>eegpt_features/features_sub-067.pt</t>
         </is>
       </c>
-      <c r="J68" t="n">
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-067.pt</t>
+        </is>
+      </c>
+      <c r="K68" t="n">
         <v>0.04359254272149751</v>
       </c>
-      <c r="K68" t="n">
+      <c r="L68" t="n">
         <v>0.1280207685118628</v>
       </c>
-      <c r="L68" t="n">
+      <c r="M68" t="n">
         <v>0.0770439470906451</v>
       </c>
-      <c r="M68" t="n">
+      <c r="N68" t="n">
         <v>0.7268164236760468</v>
       </c>
-      <c r="N68" t="n">
+      <c r="O68" t="n">
         <v>1.85809136806254</v>
       </c>
-      <c r="O68" t="n">
+      <c r="P68" t="n">
         <v>6.805889758868396</v>
       </c>
-      <c r="P68" t="n">
+      <c r="Q68" t="n">
         <v>0.2983022686810518</v>
       </c>
-      <c r="Q68" t="n">
+      <c r="R68" t="n">
         <v>1.990415824800907</v>
       </c>
     </row>
@@ -5046,28 +5386,33 @@
           <t>eegpt_features/features_sub-068.pt</t>
         </is>
       </c>
-      <c r="J69" t="n">
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-068.pt</t>
+        </is>
+      </c>
+      <c r="K69" t="n">
         <v>0.04320140676468715</v>
       </c>
-      <c r="K69" t="n">
+      <c r="L69" t="n">
         <v>0.02747741288037952</v>
       </c>
-      <c r="L69" t="n">
+      <c r="M69" t="n">
         <v>0.08433904065291072</v>
       </c>
-      <c r="M69" t="n">
+      <c r="N69" t="n">
         <v>0.8272397550824795</v>
       </c>
-      <c r="N69" t="n">
+      <c r="O69" t="n">
         <v>2.174384069981851</v>
       </c>
-      <c r="O69" t="n">
+      <c r="P69" t="n">
         <v>13.59819660687719</v>
       </c>
-      <c r="P69" t="n">
-        <v>0.318748162304203</v>
-      </c>
       <c r="Q69" t="n">
+        <v>0.3187481623042028</v>
+      </c>
+      <c r="R69" t="n">
         <v>1.469855303597616</v>
       </c>
     </row>
@@ -5113,28 +5458,33 @@
           <t>eegpt_features/features_sub-069.pt</t>
         </is>
       </c>
-      <c r="J70" t="n">
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-069.pt</t>
+        </is>
+      </c>
+      <c r="K70" t="n">
         <v>0.08944573868151562</v>
       </c>
-      <c r="K70" t="n">
+      <c r="L70" t="n">
         <v>0.0467800471287385</v>
       </c>
-      <c r="L70" t="n">
+      <c r="M70" t="n">
         <v>0.1466928644062992</v>
       </c>
-      <c r="M70" t="n">
+      <c r="N70" t="n">
         <v>0.6346549616898941</v>
       </c>
-      <c r="N70" t="n">
+      <c r="O70" t="n">
         <v>1.704699633800135</v>
       </c>
-      <c r="O70" t="n">
+      <c r="P70" t="n">
         <v>5.934722343454074</v>
       </c>
-      <c r="P70" t="n">
+      <c r="Q70" t="n">
         <v>0.2753720200722896</v>
       </c>
-      <c r="Q70" t="n">
+      <c r="R70" t="n">
         <v>1.838472592770601</v>
       </c>
     </row>
@@ -5180,28 +5530,33 @@
           <t>eegpt_features/features_sub-070.pt</t>
         </is>
       </c>
-      <c r="J71" t="n">
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-070.pt</t>
+        </is>
+      </c>
+      <c r="K71" t="n">
         <v>0.03256647389382615</v>
       </c>
-      <c r="K71" t="n">
+      <c r="L71" t="n">
         <v>0.03897133936603501</v>
       </c>
-      <c r="L71" t="n">
+      <c r="M71" t="n">
         <v>0.08679439283022154</v>
       </c>
-      <c r="M71" t="n">
+      <c r="N71" t="n">
         <v>0.822623046981614</v>
       </c>
-      <c r="N71" t="n">
+      <c r="O71" t="n">
         <v>2.723683118830438</v>
       </c>
-      <c r="O71" t="n">
+      <c r="P71" t="n">
         <v>13.44377612307457</v>
       </c>
-      <c r="P71" t="n">
-        <v>0.3732637932047339</v>
-      </c>
       <c r="Q71" t="n">
+        <v>0.373263793204734</v>
+      </c>
+      <c r="R71" t="n">
         <v>1.495372435953107</v>
       </c>
     </row>
@@ -5247,28 +5602,33 @@
           <t>eegpt_features/features_sub-071.pt</t>
         </is>
       </c>
-      <c r="J72" t="n">
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-071.pt</t>
+        </is>
+      </c>
+      <c r="K72" t="n">
         <v>0.05665378605626044</v>
       </c>
-      <c r="K72" t="n">
+      <c r="L72" t="n">
         <v>0.05670280273330607</v>
       </c>
-      <c r="L72" t="n">
+      <c r="M72" t="n">
         <v>0.09249730932348117</v>
       </c>
-      <c r="M72" t="n">
+      <c r="N72" t="n">
         <v>0.7716302640361199</v>
       </c>
-      <c r="N72" t="n">
+      <c r="O72" t="n">
         <v>1.719620356803764</v>
       </c>
-      <c r="O72" t="n">
+      <c r="P72" t="n">
         <v>7.924583065844753</v>
       </c>
-      <c r="P72" t="n">
+      <c r="Q72" t="n">
         <v>0.2887090975638203</v>
       </c>
-      <c r="Q72" t="n">
+      <c r="R72" t="n">
         <v>1.74028608697377</v>
       </c>
     </row>
@@ -5314,28 +5674,33 @@
           <t>eegpt_features/features_sub-072.pt</t>
         </is>
       </c>
-      <c r="J73" t="n">
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-072.pt</t>
+        </is>
+      </c>
+      <c r="K73" t="n">
         <v>0.03430213779039591</v>
       </c>
-      <c r="K73" t="n">
+      <c r="L73" t="n">
         <v>0.03076383400093465</v>
       </c>
-      <c r="L73" t="n">
+      <c r="M73" t="n">
         <v>0.1087413556123434</v>
       </c>
-      <c r="M73" t="n">
+      <c r="N73" t="n">
         <v>0.7993934083891725</v>
       </c>
-      <c r="N73" t="n">
+      <c r="O73" t="n">
         <v>3.170677708647625</v>
       </c>
-      <c r="O73" t="n">
+      <c r="P73" t="n">
         <v>13.97837808610226</v>
       </c>
-      <c r="P73" t="n">
-        <v>0.3416053612809933</v>
-      </c>
       <c r="Q73" t="n">
+        <v>0.3416053612809932</v>
+      </c>
+      <c r="R73" t="n">
         <v>1.521511148445845</v>
       </c>
     </row>
@@ -5381,28 +5746,33 @@
           <t>eegpt_features/features_sub-073.pt</t>
         </is>
       </c>
-      <c r="J74" t="n">
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-073.pt</t>
+        </is>
+      </c>
+      <c r="K74" t="n">
         <v>0.04311625799265997</v>
       </c>
-      <c r="K74" t="n">
+      <c r="L74" t="n">
         <v>0.02655179300656648</v>
       </c>
-      <c r="L74" t="n">
+      <c r="M74" t="n">
         <v>0.09336249018771692</v>
       </c>
-      <c r="M74" t="n">
+      <c r="N74" t="n">
         <v>0.8186303343132778</v>
       </c>
-      <c r="N74" t="n">
+      <c r="O74" t="n">
         <v>2.374022692838323</v>
       </c>
-      <c r="O74" t="n">
+      <c r="P74" t="n">
         <v>13.7712321277378</v>
       </c>
-      <c r="P74" t="n">
-        <v>0.3442093965827816</v>
-      </c>
       <c r="Q74" t="n">
+        <v>0.3442093965827818</v>
+      </c>
+      <c r="R74" t="n">
         <v>1.429966034831587</v>
       </c>
     </row>
@@ -5448,28 +5818,33 @@
           <t>eegpt_features/features_sub-074.pt</t>
         </is>
       </c>
-      <c r="J75" t="n">
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-074.pt</t>
+        </is>
+      </c>
+      <c r="K75" t="n">
         <v>0.04558809471031074</v>
       </c>
-      <c r="K75" t="n">
+      <c r="L75" t="n">
         <v>0.02943715437082221</v>
       </c>
-      <c r="L75" t="n">
+      <c r="M75" t="n">
         <v>0.09258314419057455</v>
       </c>
-      <c r="M75" t="n">
+      <c r="N75" t="n">
         <v>0.8128920549479028</v>
       </c>
-      <c r="N75" t="n">
+      <c r="O75" t="n">
         <v>2.262475225217244</v>
       </c>
-      <c r="O75" t="n">
+      <c r="P75" t="n">
         <v>12.81151232688596</v>
       </c>
-      <c r="P75" t="n">
+      <c r="Q75" t="n">
         <v>0.3325523837890013</v>
       </c>
-      <c r="Q75" t="n">
+      <c r="R75" t="n">
         <v>1.528055199912915</v>
       </c>
     </row>
@@ -5515,28 +5890,33 @@
           <t>eegpt_features/features_sub-075.pt</t>
         </is>
       </c>
-      <c r="J76" t="n">
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-075.pt</t>
+        </is>
+      </c>
+      <c r="K76" t="n">
         <v>0.06876416119020352</v>
       </c>
-      <c r="K76" t="n">
+      <c r="L76" t="n">
         <v>0.06573654719265701</v>
       </c>
-      <c r="L76" t="n">
+      <c r="M76" t="n">
         <v>0.08852581032490479</v>
       </c>
-      <c r="M76" t="n">
+      <c r="N76" t="n">
         <v>0.7518287541582506</v>
       </c>
-      <c r="N76" t="n">
+      <c r="O76" t="n">
         <v>1.688708284490514</v>
       </c>
-      <c r="O76" t="n">
+      <c r="P76" t="n">
         <v>7.6467498159206</v>
       </c>
-      <c r="P76" t="n">
-        <v>0.2729124542140111</v>
-      </c>
       <c r="Q76" t="n">
+        <v>0.272912454214011</v>
+      </c>
+      <c r="R76" t="n">
         <v>1.821345477301449</v>
       </c>
     </row>
@@ -5582,28 +5962,33 @@
           <t>eegpt_features/features_sub-076.pt</t>
         </is>
       </c>
-      <c r="J77" t="n">
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-076.pt</t>
+        </is>
+      </c>
+      <c r="K77" t="n">
         <v>0.03197550832577323</v>
       </c>
-      <c r="K77" t="n">
+      <c r="L77" t="n">
         <v>0.04936041413794795</v>
       </c>
-      <c r="L77" t="n">
+      <c r="M77" t="n">
         <v>0.08374087777452976</v>
       </c>
-      <c r="M77" t="n">
+      <c r="N77" t="n">
         <v>0.8155745221033966</v>
       </c>
-      <c r="N77" t="n">
+      <c r="O77" t="n">
         <v>2.634205808028649</v>
       </c>
-      <c r="O77" t="n">
+      <c r="P77" t="n">
         <v>11.40710531558002</v>
       </c>
-      <c r="P77" t="n">
+      <c r="Q77" t="n">
         <v>0.3540459726022707</v>
       </c>
-      <c r="Q77" t="n">
+      <c r="R77" t="n">
         <v>1.612546286421722</v>
       </c>
     </row>
@@ -5649,28 +6034,33 @@
           <t>eegpt_features/features_sub-077.pt</t>
         </is>
       </c>
-      <c r="J78" t="n">
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-077.pt</t>
+        </is>
+      </c>
+      <c r="K78" t="n">
         <v>0.02712138187973041</v>
       </c>
-      <c r="K78" t="n">
+      <c r="L78" t="n">
         <v>0.03192480589846822</v>
       </c>
-      <c r="L78" t="n">
+      <c r="M78" t="n">
         <v>0.08215133853925558</v>
       </c>
-      <c r="M78" t="n">
+      <c r="N78" t="n">
         <v>0.842727934905506</v>
       </c>
-      <c r="N78" t="n">
+      <c r="O78" t="n">
         <v>3.049258553788665</v>
       </c>
-      <c r="O78" t="n">
+      <c r="P78" t="n">
         <v>16.1790098783916</v>
       </c>
-      <c r="P78" t="n">
-        <v>0.4033842437901424</v>
-      </c>
       <c r="Q78" t="n">
+        <v>0.4033842437901427</v>
+      </c>
+      <c r="R78" t="n">
         <v>1.452326109451137</v>
       </c>
     </row>
@@ -5716,28 +6106,33 @@
           <t>eegpt_features/features_sub-078.pt</t>
         </is>
       </c>
-      <c r="J79" t="n">
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-078.pt</t>
+        </is>
+      </c>
+      <c r="K79" t="n">
         <v>0.02813477121093115</v>
       </c>
-      <c r="K79" t="n">
+      <c r="L79" t="n">
         <v>0.03323293236359877</v>
       </c>
-      <c r="L79" t="n">
+      <c r="M79" t="n">
         <v>0.08214391521051566</v>
       </c>
-      <c r="M79" t="n">
+      <c r="N79" t="n">
         <v>0.8403878685109997</v>
       </c>
-      <c r="N79" t="n">
+      <c r="O79" t="n">
         <v>2.945472972372636</v>
       </c>
-      <c r="O79" t="n">
+      <c r="P79" t="n">
         <v>15.52901102929658</v>
       </c>
-      <c r="P79" t="n">
+      <c r="Q79" t="n">
         <v>0.3936498997365088</v>
       </c>
-      <c r="Q79" t="n">
+      <c r="R79" t="n">
         <v>1.441533600846581</v>
       </c>
     </row>
@@ -5783,28 +6178,33 @@
           <t>eegpt_features/features_sub-079.pt</t>
         </is>
       </c>
-      <c r="J80" t="n">
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-079.pt</t>
+        </is>
+      </c>
+      <c r="K80" t="n">
         <v>0.04915482193823752</v>
       </c>
-      <c r="K80" t="n">
+      <c r="L80" t="n">
         <v>0.05849886518604375</v>
       </c>
-      <c r="L80" t="n">
+      <c r="M80" t="n">
         <v>0.08380769346387397</v>
       </c>
-      <c r="M80" t="n">
+      <c r="N80" t="n">
         <v>0.7897347575486293</v>
       </c>
-      <c r="N80" t="n">
+      <c r="O80" t="n">
         <v>2.015404718846078</v>
       </c>
-      <c r="O80" t="n">
+      <c r="P80" t="n">
         <v>9.786494276326001</v>
       </c>
-      <c r="P80" t="n">
+      <c r="Q80" t="n">
         <v>0.2999921487075699</v>
       </c>
-      <c r="Q80" t="n">
+      <c r="R80" t="n">
         <v>1.691390024944595</v>
       </c>
     </row>
@@ -5850,28 +6250,33 @@
           <t>eegpt_features/features_sub-080.pt</t>
         </is>
       </c>
-      <c r="J81" t="n">
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-080.pt</t>
+        </is>
+      </c>
+      <c r="K81" t="n">
         <v>0.1213328500804824</v>
       </c>
-      <c r="K81" t="n">
+      <c r="L81" t="n">
         <v>0.04456407412727693</v>
       </c>
-      <c r="L81" t="n">
+      <c r="M81" t="n">
         <v>0.08033852375007033</v>
       </c>
-      <c r="M81" t="n">
+      <c r="N81" t="n">
         <v>0.7349054933418855</v>
       </c>
-      <c r="N81" t="n">
+      <c r="O81" t="n">
         <v>1.225388908883114</v>
       </c>
-      <c r="O81" t="n">
+      <c r="P81" t="n">
         <v>7.317172339294845</v>
       </c>
-      <c r="P81" t="n">
+      <c r="Q81" t="n">
         <v>0.3174620264989785</v>
       </c>
-      <c r="Q81" t="n">
+      <c r="R81" t="n">
         <v>1.682813442417092</v>
       </c>
     </row>
@@ -5917,28 +6322,33 @@
           <t>eegpt_features/features_sub-081.pt</t>
         </is>
       </c>
-      <c r="J82" t="n">
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-081.pt</t>
+        </is>
+      </c>
+      <c r="K82" t="n">
         <v>0.0336085927356661</v>
       </c>
-      <c r="K82" t="n">
+      <c r="L82" t="n">
         <v>0.02535262755112455</v>
       </c>
-      <c r="L82" t="n">
+      <c r="M82" t="n">
         <v>0.09444694412991728</v>
       </c>
-      <c r="M82" t="n">
+      <c r="N82" t="n">
         <v>0.8265293054513506</v>
       </c>
-      <c r="N82" t="n">
+      <c r="O82" t="n">
         <v>2.859161970785277</v>
       </c>
-      <c r="O82" t="n">
+      <c r="P82" t="n">
         <v>15.76163651060444</v>
       </c>
-      <c r="P82" t="n">
-        <v>0.3739439106213681</v>
-      </c>
       <c r="Q82" t="n">
+        <v>0.373943910621368</v>
+      </c>
+      <c r="R82" t="n">
         <v>1.404026408105289</v>
       </c>
     </row>
@@ -5984,28 +6394,33 @@
           <t>eegpt_features/features_sub-082.pt</t>
         </is>
       </c>
-      <c r="J83" t="n">
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-082.pt</t>
+        </is>
+      </c>
+      <c r="K83" t="n">
         <v>0.04861822986041959</v>
       </c>
-      <c r="K83" t="n">
+      <c r="L83" t="n">
         <v>0.03180919027978459</v>
       </c>
-      <c r="L83" t="n">
+      <c r="M83" t="n">
         <v>0.0884386744919881</v>
       </c>
-      <c r="M83" t="n">
+      <c r="N83" t="n">
         <v>0.8129457002285472</v>
       </c>
-      <c r="N83" t="n">
+      <c r="O83" t="n">
         <v>2.078324827135893</v>
       </c>
-      <c r="O83" t="n">
+      <c r="P83" t="n">
         <v>11.92830654556456</v>
       </c>
-      <c r="P83" t="n">
+      <c r="Q83" t="n">
         <v>0.31516355915529</v>
       </c>
-      <c r="Q83" t="n">
+      <c r="R83" t="n">
         <v>1.506600249032049</v>
       </c>
     </row>
@@ -6051,28 +6466,33 @@
           <t>eegpt_features/features_sub-083.pt</t>
         </is>
       </c>
-      <c r="J84" t="n">
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-083.pt</t>
+        </is>
+      </c>
+      <c r="K84" t="n">
         <v>0.02804065463476636</v>
       </c>
-      <c r="K84" t="n">
+      <c r="L84" t="n">
         <v>0.02683253556892766</v>
       </c>
-      <c r="L84" t="n">
+      <c r="M84" t="n">
         <v>0.08699571204164515</v>
       </c>
-      <c r="M84" t="n">
+      <c r="N84" t="n">
         <v>0.8404948631648013</v>
       </c>
-      <c r="N84" t="n">
+      <c r="O84" t="n">
         <v>3.109831315589537</v>
       </c>
-      <c r="O84" t="n">
+      <c r="P84" t="n">
         <v>17.04214449191675</v>
       </c>
-      <c r="P84" t="n">
+      <c r="Q84" t="n">
         <v>0.4256032589456474</v>
       </c>
-      <c r="Q84" t="n">
+      <c r="R84" t="n">
         <v>1.408933361467178</v>
       </c>
     </row>
@@ -6118,28 +6538,33 @@
           <t>eegpt_features/features_sub-084.pt</t>
         </is>
       </c>
-      <c r="J85" t="n">
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-084.pt</t>
+        </is>
+      </c>
+      <c r="K85" t="n">
         <v>0.03876430570640337</v>
       </c>
-      <c r="K85" t="n">
+      <c r="L85" t="n">
         <v>0.03956196764985421</v>
       </c>
-      <c r="L85" t="n">
+      <c r="M85" t="n">
         <v>0.1223242407957503</v>
       </c>
-      <c r="M85" t="n">
+      <c r="N85" t="n">
         <v>0.7746706745217948</v>
       </c>
-      <c r="N85" t="n">
+      <c r="O85" t="n">
         <v>3.189289019148382</v>
       </c>
-      <c r="O85" t="n">
+      <c r="P85" t="n">
         <v>11.53869798443629</v>
       </c>
-      <c r="P85" t="n">
-        <v>0.3720263441744064</v>
-      </c>
       <c r="Q85" t="n">
+        <v>0.3720263441744063</v>
+      </c>
+      <c r="R85" t="n">
         <v>1.616238358308277</v>
       </c>
     </row>
@@ -6185,28 +6610,33 @@
           <t>eegpt_features/features_sub-085.pt</t>
         </is>
       </c>
-      <c r="J86" t="n">
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-085.pt</t>
+        </is>
+      </c>
+      <c r="K86" t="n">
         <v>0.02828419935279606</v>
       </c>
-      <c r="K86" t="n">
+      <c r="L86" t="n">
         <v>0.04347232038565296</v>
       </c>
-      <c r="L86" t="n">
+      <c r="M86" t="n">
         <v>0.1047162896567327</v>
       </c>
-      <c r="M86" t="n">
+      <c r="N86" t="n">
         <v>0.8047661393573101</v>
       </c>
-      <c r="N86" t="n">
+      <c r="O86" t="n">
         <v>3.724838170658163</v>
       </c>
-      <c r="O86" t="n">
+      <c r="P86" t="n">
         <v>13.68272717597483</v>
       </c>
-      <c r="P86" t="n">
-        <v>0.3892762995434191</v>
-      </c>
       <c r="Q86" t="n">
+        <v>0.389276299543419</v>
+      </c>
+      <c r="R86" t="n">
         <v>1.726450888207953</v>
       </c>
     </row>
@@ -6252,28 +6682,33 @@
           <t>eegpt_features/features_sub-086.pt</t>
         </is>
       </c>
-      <c r="J87" t="n">
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-086.pt</t>
+        </is>
+      </c>
+      <c r="K87" t="n">
         <v>0.04293599041133043</v>
       </c>
-      <c r="K87" t="n">
+      <c r="L87" t="n">
         <v>0.06761093722983003</v>
       </c>
-      <c r="L87" t="n">
+      <c r="M87" t="n">
         <v>0.07337191605822535</v>
       </c>
-      <c r="M87" t="n">
+      <c r="N87" t="n">
         <v>0.7975932263991428</v>
       </c>
-      <c r="N87" t="n">
+      <c r="O87" t="n">
         <v>1.986805995918724</v>
       </c>
-      <c r="O87" t="n">
+      <c r="P87" t="n">
         <v>9.368369656341784</v>
       </c>
-      <c r="P87" t="n">
-        <v>0.2717290873994827</v>
-      </c>
       <c r="Q87" t="n">
+        <v>0.2717290873994829</v>
+      </c>
+      <c r="R87" t="n">
         <v>1.887165255401384</v>
       </c>
     </row>
@@ -6319,28 +6754,33 @@
           <t>eegpt_features/features_sub-087.pt</t>
         </is>
       </c>
-      <c r="J88" t="n">
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-087.pt</t>
+        </is>
+      </c>
+      <c r="K88" t="n">
         <v>0.03616613242135856</v>
       </c>
-      <c r="K88" t="n">
+      <c r="L88" t="n">
         <v>0.02885591330980674</v>
       </c>
-      <c r="L88" t="n">
+      <c r="M88" t="n">
         <v>0.0871946374026981</v>
       </c>
-      <c r="M88" t="n">
+      <c r="N88" t="n">
         <v>0.8301910451777627</v>
       </c>
-      <c r="N88" t="n">
+      <c r="O88" t="n">
         <v>2.720875481693625</v>
       </c>
-      <c r="O88" t="n">
+      <c r="P88" t="n">
         <v>15.21485950434592</v>
       </c>
-      <c r="P88" t="n">
-        <v>0.3235866608726252</v>
-      </c>
       <c r="Q88" t="n">
+        <v>0.3235866608726253</v>
+      </c>
+      <c r="R88" t="n">
         <v>1.455504336959076</v>
       </c>
     </row>
@@ -6386,28 +6826,33 @@
           <t>eegpt_features/features_sub-088.pt</t>
         </is>
       </c>
-      <c r="J89" t="n">
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>eegpt_features/small_features_sub-088.pt</t>
+        </is>
+      </c>
+      <c r="K89" t="n">
         <v>0.06579694653442568</v>
       </c>
-      <c r="K89" t="n">
+      <c r="L89" t="n">
         <v>0.04403093253622747</v>
       </c>
-      <c r="L89" t="n">
+      <c r="M89" t="n">
         <v>0.09268563770386082</v>
       </c>
-      <c r="M89" t="n">
+      <c r="N89" t="n">
         <v>0.7716500121611191</v>
       </c>
-      <c r="N89" t="n">
+      <c r="O89" t="n">
         <v>1.665466276302744</v>
       </c>
-      <c r="O89" t="n">
+      <c r="P89" t="n">
         <v>8.653634627071588</v>
       </c>
-      <c r="P89" t="n">
-        <v>0.2847214305169611</v>
-      </c>
       <c r="Q89" t="n">
+        <v>0.284721430516961</v>
+      </c>
+      <c r="R89" t="n">
         <v>1.640486475904775</v>
       </c>
     </row>

</xml_diff>